<commit_message>
docs: borrow atlas quick links and contents panel
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R82b6380e0935403a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R11c7113b031a44a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R650c6a97b6004efa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R5ae8c99cd4284014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R18dd3bdf0b78482d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R20e7284039b04ae6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rb933b022e3ae4a5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Re83a0e109a674f49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -847,7 +847,7 @@
         <x:v>The hero should use the private playbook cover art as a background with layered dark overlays and ATLAS-style accent treatment.</x:v>
       </x:c>
       <x:c r="I5" s="14" t="str">
-        <x:v>Code inspection shows the hero background uses url(\./cover.png\) with additional gradients, scan-line overlays, and orange-to-magenta accent lighting.</x:v>
+        <x:v>Code inspection shows the hero background uses ./cover.png with additional gradients, scan-line overlays, and orange-to-magenta accent lighting.</x:v>
       </x:c>
       <x:c r="J5" s="14" t="str">
         <x:v>Verified</x:v>
@@ -1264,13 +1264,13 @@
         <x:v>F-010</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>Public Tracker Workbook Output</x:v>
+        <x:v>Public Tracker And Report Outputs</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
         <x:v>Repo Deliverable</x:v>
       </x:c>
       <x:c r="D11" s="14" t="str">
-        <x:v>README.md, feature_status_tracker.csv, feature_status_tracker.xlsx</x:v>
+        <x:v>README.md, feature_status_tracker.csv, feature_status_tracker.xlsx, feature_qa_report.md</x:v>
       </x:c>
       <x:c r="E11" s="14" t="str">
         <x:v>Repo root tracker artifacts</x:v>
@@ -1279,13 +1279,13 @@
         <x:v>Repo operator</x:v>
       </x:c>
       <x:c r="G11" s="14" t="str">
-        <x:v>As a repo operator, I want the QA skill to leave a workbook output in the audited repo so that the tracker is available as both a canonical CSV and a richer spreadsheet view.</x:v>
+        <x:v>As a repo operator, I want the QA skill to leave tracker, workbook, and final report outputs in the audited repo so that the repo contains the full audit artifact set.</x:v>
       </x:c>
       <x:c r="H11" s="14" t="str">
-        <x:v>The audited repo should contain feature_status_tracker.csv as the source of truth and feature_status_tracker.xlsx as the workbook view, with README documenting both outputs.</x:v>
+        <x:v>The audited repo should contain feature_status_tracker.csv as the source of truth, feature_status_tracker.xlsx as the workbook view, and feature_qa_report.md as the final summary, with README documenting those outputs.</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>Code inspection confirms feature_status_tracker.xlsx exists at repo root and README includes a Public Tracker Outputs section listing both tracker files.</x:v>
+        <x:v>Code inspection confirms feature_status_tracker.xlsx and feature_qa_report.md exist at repo root and README includes a Public Tracker Outputs section listing the audit artifacts.</x:v>
       </x:c>
       <x:c r="J11" s="14" t="str">
         <x:v>Verified</x:v>
@@ -1294,10 +1294,10 @@
         <x:v>Code inspection</x:v>
       </x:c>
       <x:c r="L11" s="14" t="str">
-        <x:v>Confirm feature_status_tracker.xlsx exists at the repo root and inspect README.md for the tracker outputs section.</x:v>
+        <x:v>Confirm feature_status_tracker.xlsx and feature_qa_report.md exist at the repo root and inspect README.md for the tracker outputs section.</x:v>
       </x:c>
       <x:c r="M11" s="14" t="str">
-        <x:v>Pass - workbook artifact exists and the README exposes both tracker outputs.</x:v>
+        <x:v>Pass - workbook and report artifacts exist and the README exposes the audit outputs.</x:v>
       </x:c>
       <x:c r="N11" s="14" t="str"/>
       <x:c r="O11" s="14" t="str">
@@ -1308,16 +1308,16 @@
       </x:c>
       <x:c r="Q11" s="14" t="str"/>
       <x:c r="R11" s="14" t="str">
-        <x:v>README.md, feature_status_tracker.csv, feature_status_tracker.xlsx</x:v>
+        <x:v>README.md, feature_status_tracker.csv, feature_status_tracker.xlsx, feature_qa_report.md</x:v>
       </x:c>
       <x:c r="S11" s="14" t="str">
-        <x:v>Pending current pass commit</x:v>
+        <x:v>e2fa4c7</x:v>
       </x:c>
       <x:c r="T11" s="14" t="str">
-        <x:v>Regenerate workbook after tracker update and confirm the dashboard still renders tracked rows.</x:v>
+        <x:v>Regenerate workbook and report after tracker update and confirm the dashboard plus report parse cleanly.</x:v>
       </x:c>
       <x:c r="U11" s="14" t="str">
-        <x:v>Pass - workbook regenerated from the updated tracker with no formula errors.</x:v>
+        <x:v>Pass - workbook regenerated from the updated tracker with no formula errors and the final report regenerated cleanly from the CSV.</x:v>
       </x:c>
       <x:c r="V11" s="14" t="str">
         <x:v>Verified</x:v>
@@ -1326,65 +1326,157 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="X11" s="14" t="str">
-        <x:v>Workbook generated by the repo skill builder against the public repo root.</x:v>
+        <x:v>Workbook and report were generated by the repo skill tooling against the public repo root.</x:v>
       </x:c>
       <x:c r="Y11" s="14" t="str">
         <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
-      <x:c r="A12" s="14"/>
-      <x:c r="B12" s="14"/>
-      <x:c r="C12" s="14"/>
-      <x:c r="D12" s="14"/>
-      <x:c r="E12" s="14"/>
-      <x:c r="F12" s="14"/>
-      <x:c r="G12" s="14"/>
-      <x:c r="H12" s="14"/>
-      <x:c r="I12" s="14"/>
-      <x:c r="J12" s="14"/>
-      <x:c r="K12" s="14"/>
-      <x:c r="L12" s="14"/>
-      <x:c r="M12" s="14"/>
-      <x:c r="N12" s="14"/>
-      <x:c r="O12" s="14"/>
-      <x:c r="P12" s="14"/>
-      <x:c r="Q12" s="14"/>
-      <x:c r="R12" s="14"/>
-      <x:c r="S12" s="14"/>
-      <x:c r="T12" s="14"/>
-      <x:c r="U12" s="14"/>
-      <x:c r="V12" s="14"/>
-      <x:c r="W12" s="14"/>
-      <x:c r="X12" s="14"/>
-      <x:c r="Y12" s="14"/>
+      <x:c r="A12" s="14" t="str">
+        <x:v>F-011</x:v>
+      </x:c>
+      <x:c r="B12" s="14" t="str">
+        <x:v>Agent Surface Quick Links</x:v>
+      </x:c>
+      <x:c r="C12" s="14" t="str">
+        <x:v>Hero / Navigation</x:v>
+      </x:c>
+      <x:c r="D12" s="14" t="str">
+        <x:v>index.html</x:v>
+      </x:c>
+      <x:c r="E12" s="14" t="str">
+        <x:v>Hero agent-links strip</x:v>
+      </x:c>
+      <x:c r="F12" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G12" s="14" t="str">
+        <x:v>As a visitor, I want to see the supported agent surfaces immediately so that I understand where ATLAS-7 fits into actual workflows.</x:v>
+      </x:c>
+      <x:c r="H12" s="14" t="str">
+        <x:v>The hero should include a quick-link strip highlighting Claude Code, Codex, Cursor, and Grok Build, linking back to the public ATLAS Codex page.</x:v>
+      </x:c>
+      <x:c r="I12" s="14" t="str">
+        <x:v>Code inspection confirms an agent-links row under the hero CTAs with four labeled links, each pointing to the public ATLAS Codex page in a new tab.</x:v>
+      </x:c>
+      <x:c r="J12" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K12" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L12" s="14" t="str">
+        <x:v>Inspect the agent-links row in index.html and confirm the labels, targets, and placement beneath the main hero CTAs.</x:v>
+      </x:c>
+      <x:c r="M12" s="14" t="str">
+        <x:v>Pass - the supported agent surfaces are visible and linked from the hero.</x:v>
+      </x:c>
+      <x:c r="N12" s="14" t="str"/>
+      <x:c r="O12" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P12" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q12" s="14" t="str"/>
+      <x:c r="R12" s="14" t="str">
+        <x:v>index.html</x:v>
+      </x:c>
+      <x:c r="S12" s="14" t="str">
+        <x:v>Pending current pass commit</x:v>
+      </x:c>
+      <x:c r="T12" s="14" t="str">
+        <x:v>Regenerate workbook and report after tracker update and confirm the new row is reflected in repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U12" s="14" t="str">
+        <x:v>Pending current pass rerun.</x:v>
+      </x:c>
+      <x:c r="V12" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W12" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X12" s="14" t="str">
+        <x:v>Borrowed from the ATLAS Codex front-page quick-link pattern.</x:v>
+      </x:c>
+      <x:c r="Y12" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
-      <x:c r="A13" s="14"/>
-      <x:c r="B13" s="14"/>
-      <x:c r="C13" s="14"/>
-      <x:c r="D13" s="14"/>
-      <x:c r="E13" s="14"/>
-      <x:c r="F13" s="14"/>
-      <x:c r="G13" s="14"/>
-      <x:c r="H13" s="14"/>
-      <x:c r="I13" s="14"/>
-      <x:c r="J13" s="14"/>
-      <x:c r="K13" s="14"/>
-      <x:c r="L13" s="14"/>
-      <x:c r="M13" s="14"/>
-      <x:c r="N13" s="14"/>
-      <x:c r="O13" s="14"/>
-      <x:c r="P13" s="14"/>
-      <x:c r="Q13" s="14"/>
-      <x:c r="R13" s="14"/>
-      <x:c r="S13" s="14"/>
-      <x:c r="T13" s="14"/>
-      <x:c r="U13" s="14"/>
-      <x:c r="V13" s="14"/>
-      <x:c r="W13" s="14"/>
-      <x:c r="X13" s="14"/>
-      <x:c r="Y13" s="14"/>
+      <x:c r="A13" s="14" t="str">
+        <x:v>F-012</x:v>
+      </x:c>
+      <x:c r="B13" s="14" t="str">
+        <x:v>Contents Jump Panel</x:v>
+      </x:c>
+      <x:c r="C13" s="14" t="str">
+        <x:v>Hero / Navigation</x:v>
+      </x:c>
+      <x:c r="D13" s="14" t="str">
+        <x:v>index.html</x:v>
+      </x:c>
+      <x:c r="E13" s="14" t="str">
+        <x:v>Hero contents panel with section anchors</x:v>
+      </x:c>
+      <x:c r="F13" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G13" s="14" t="str">
+        <x:v>As a visitor, I want quick section jumps near the hero so that I can move directly to the parts of the public page I care about.</x:v>
+      </x:c>
+      <x:c r="H13" s="14" t="str">
+        <x:v>The page should include a contents panel with links to What You Get, Access Flow, Private Areas, and Public Changelog, and those destination sections should expose matching ids.</x:v>
+      </x:c>
+      <x:c r="I13" s="14" t="str">
+        <x:v>Code inspection confirms a toc-panel below the hero layout with four anchor links and matching section ids on the destination sections.</x:v>
+      </x:c>
+      <x:c r="J13" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K13" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L13" s="14" t="str">
+        <x:v>Inspect the toc-panel markup and confirm the four anchor links and corresponding section ids exist in index.html.</x:v>
+      </x:c>
+      <x:c r="M13" s="14" t="str">
+        <x:v>Pass - the contents jump panel is present and wired to the expected sections.</x:v>
+      </x:c>
+      <x:c r="N13" s="14" t="str"/>
+      <x:c r="O13" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P13" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q13" s="14" t="str"/>
+      <x:c r="R13" s="14" t="str">
+        <x:v>index.html</x:v>
+      </x:c>
+      <x:c r="S13" s="14" t="str">
+        <x:v>Pending current pass commit</x:v>
+      </x:c>
+      <x:c r="T13" s="14" t="str">
+        <x:v>Regenerate workbook and report after tracker update and confirm the new row is reflected in repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U13" s="14" t="str">
+        <x:v>Pending current pass rerun.</x:v>
+      </x:c>
+      <x:c r="V13" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W13" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X13" s="14" t="str">
+        <x:v>Borrowed from the ATLAS Codex front-page contents-panel pattern.</x:v>
+      </x:c>
+      <x:c r="Y13" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="14"/>
@@ -11897,7 +11989,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -11913,7 +12005,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -11977,14 +12069,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): finalize borrowed atlas patterns
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R18dd3bdf0b78482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R20e7284039b04ae6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rb933b022e3ae4a5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Re83a0e109a674f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rf085d35978d641b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R7797b3a157104c31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R2ecf274276004b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rc59ac50c92104612"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1384,13 +1384,13 @@
         <x:v>index.html</x:v>
       </x:c>
       <x:c r="S12" s="14" t="str">
-        <x:v>Pending current pass commit</x:v>
+        <x:v>6cce475</x:v>
       </x:c>
       <x:c r="T12" s="14" t="str">
         <x:v>Regenerate workbook and report after tracker update and confirm the new row is reflected in repo QA outputs.</x:v>
       </x:c>
       <x:c r="U12" s="14" t="str">
-        <x:v>Pending current pass rerun.</x:v>
+        <x:v>Pass - workbook and report regenerated successfully after adding the quick-link row.</x:v>
       </x:c>
       <x:c r="V12" s="14" t="str">
         <x:v>Verified</x:v>
@@ -1457,13 +1457,13 @@
         <x:v>index.html</x:v>
       </x:c>
       <x:c r="S13" s="14" t="str">
-        <x:v>Pending current pass commit</x:v>
+        <x:v>6cce475</x:v>
       </x:c>
       <x:c r="T13" s="14" t="str">
         <x:v>Regenerate workbook and report after tracker update and confirm the new row is reflected in repo QA outputs.</x:v>
       </x:c>
       <x:c r="U13" s="14" t="str">
-        <x:v>Pending current pass rerun.</x:v>
+        <x:v>Pass - workbook and report regenerated successfully after adding the contents jump panel.</x:v>
       </x:c>
       <x:c r="V13" s="14" t="str">
         <x:v>Verified</x:v>

</xml_diff>

<commit_message>
docs: clarify public join instructions
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rf085d35978d641b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R7797b3a157104c31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R2ecf274276004b97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rc59ac50c92104612"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rc79d64f4805c4c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5d8e7b33400149cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R331869f11598464d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rd4e1850468074f53"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1479,31 +1479,77 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
-      <x:c r="A14" s="14"/>
-      <x:c r="B14" s="14"/>
-      <x:c r="C14" s="14"/>
-      <x:c r="D14" s="14"/>
-      <x:c r="E14" s="14"/>
-      <x:c r="F14" s="14"/>
-      <x:c r="G14" s="14"/>
-      <x:c r="H14" s="14"/>
-      <x:c r="I14" s="14"/>
-      <x:c r="J14" s="14"/>
-      <x:c r="K14" s="14"/>
-      <x:c r="L14" s="14"/>
-      <x:c r="M14" s="14"/>
-      <x:c r="N14" s="14"/>
-      <x:c r="O14" s="14"/>
-      <x:c r="P14" s="14"/>
-      <x:c r="Q14" s="14"/>
-      <x:c r="R14" s="14"/>
-      <x:c r="S14" s="14"/>
-      <x:c r="T14" s="14"/>
-      <x:c r="U14" s="14"/>
-      <x:c r="V14" s="14"/>
-      <x:c r="W14" s="14"/>
-      <x:c r="X14" s="14"/>
-      <x:c r="Y14" s="14"/>
+      <x:c r="A14" s="14" t="str">
+        <x:v>F-013</x:v>
+      </x:c>
+      <x:c r="B14" s="14" t="str">
+        <x:v>Explicit Join Instructions</x:v>
+      </x:c>
+      <x:c r="C14" s="14" t="str">
+        <x:v>Membership / Access</x:v>
+      </x:c>
+      <x:c r="D14" s="14" t="str">
+        <x:v>index.html, README.md</x:v>
+      </x:c>
+      <x:c r="E14" s="14" t="str">
+        <x:v>Hero join strip, hero access panel, access-flow panel, README access section</x:v>
+      </x:c>
+      <x:c r="F14" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G14" s="14" t="str">
+        <x:v>As a prospective member, I want explicit join instructions so that I know exactly how to move from the public repo to private GitHub access.</x:v>
+      </x:c>
+      <x:c r="H14" s="14" t="str">
+        <x:v>The public repo should expose a clear three-step join path, explain that current Alpha members can skip straight to the GitHub handoff, and repeat that instruction in the README.</x:v>
+      </x:c>
+      <x:c r="I14" s="14" t="str">
+        <x:v>Code inspection confirms the landing page now includes a hero join strip, a dedicated three-step access panel, clarified access-flow copy, and the README access section now presents the same sequence.</x:v>
+      </x:c>
+      <x:c r="J14" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K14" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L14" s="14" t="str">
+        <x:v>Inspect the join-strip, hero access steps, and access-flow copy in index.html, then inspect the Access section in README.md for the same explicit join path.</x:v>
+      </x:c>
+      <x:c r="M14" s="14" t="str">
+        <x:v>Pass - the public repo now gives a concrete join path for both new and existing Alpha members.</x:v>
+      </x:c>
+      <x:c r="N14" s="14" t="str"/>
+      <x:c r="O14" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P14" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q14" s="14" t="str"/>
+      <x:c r="R14" s="14" t="str">
+        <x:v>index.html, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S14" s="14" t="str">
+        <x:v>Pending current pass commit</x:v>
+      </x:c>
+      <x:c r="T14" s="14" t="str">
+        <x:v>Regenerate workbook and report after adding the new access row and confirm the repo QA outputs reflect the updated join flow.</x:v>
+      </x:c>
+      <x:c r="U14" s="14" t="str">
+        <x:v>Pending current pass verification</x:v>
+      </x:c>
+      <x:c r="V14" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W14" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X14" s="14" t="str">
+        <x:v>This row captures the explicit public join instructions requested in the latest improvement pass.</x:v>
+      </x:c>
+      <x:c r="Y14" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="14"/>
@@ -11989,7 +12035,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12005,7 +12051,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12069,14 +12115,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record join-flow pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rc79d64f4805c4c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5d8e7b33400149cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R331869f11598464d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rd4e1850468074f53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R4ee7044831ae4248"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9e5bf91818014ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R9616d7eb25fc41a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rfd3b7caa5a304e89"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1530,13 +1530,13 @@
         <x:v>index.html, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
       </x:c>
       <x:c r="S14" s="14" t="str">
-        <x:v>Pending current pass commit</x:v>
+        <x:v>f583766</x:v>
       </x:c>
       <x:c r="T14" s="14" t="str">
         <x:v>Regenerate workbook and report after adding the new access row and confirm the repo QA outputs reflect the updated join flow.</x:v>
       </x:c>
       <x:c r="U14" s="14" t="str">
-        <x:v>Pending current pass verification</x:v>
+        <x:v>Pass - workbook and report regenerated successfully after the join-flow clarification pass.</x:v>
       </x:c>
       <x:c r="V14" s="14" t="str">
         <x:v>Verified</x:v>

</xml_diff>

<commit_message>
docs(qa): record atlas codex link pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R4ee7044831ae4248"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9e5bf91818014ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R9616d7eb25fc41a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rfd3b7caa5a304e89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R34e0d36c7b734ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R6a7edaae2a4e4bc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rd7938a3e753c46f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rca04b716f2f54aee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1552,31 +1552,77 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
-      <x:c r="A15" s="14"/>
-      <x:c r="B15" s="14"/>
-      <x:c r="C15" s="14"/>
-      <x:c r="D15" s="14"/>
-      <x:c r="E15" s="14"/>
-      <x:c r="F15" s="14"/>
-      <x:c r="G15" s="14"/>
-      <x:c r="H15" s="14"/>
-      <x:c r="I15" s="14"/>
-      <x:c r="J15" s="14"/>
-      <x:c r="K15" s="14"/>
-      <x:c r="L15" s="14"/>
-      <x:c r="M15" s="14"/>
-      <x:c r="N15" s="14"/>
-      <x:c r="O15" s="14"/>
-      <x:c r="P15" s="14"/>
-      <x:c r="Q15" s="14"/>
-      <x:c r="R15" s="14"/>
-      <x:c r="S15" s="14"/>
-      <x:c r="T15" s="14"/>
-      <x:c r="U15" s="14"/>
-      <x:c r="V15" s="14"/>
-      <x:c r="W15" s="14"/>
-      <x:c r="X15" s="14"/>
-      <x:c r="Y15" s="14"/>
+      <x:c r="A15" s="14" t="str">
+        <x:v>F-014</x:v>
+      </x:c>
+      <x:c r="B15" s="14" t="str">
+        <x:v>ATLAS Codex Public Page CTA</x:v>
+      </x:c>
+      <x:c r="C15" s="14" t="str">
+        <x:v>Hero / External Navigation</x:v>
+      </x:c>
+      <x:c r="D15" s="14" t="str">
+        <x:v>src/app.js, index.html, README.md</x:v>
+      </x:c>
+      <x:c r="E15" s="14" t="str">
+        <x:v>Hero CTA row, access-flow helper copy, README public demo section</x:v>
+      </x:c>
+      <x:c r="F15" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G15" s="14" t="str">
+        <x:v>As a visitor, I want a direct link to the public ATLAS Codex page so that I can inspect the live public agent surface before deciding whether to join the private repo.</x:v>
+      </x:c>
+      <x:c r="H15" s="14" t="str">
+        <x:v>The landing page should expose a clear CTA to the public ATLAS Codex page in the hero flow, repeat that link in the access section, and document it in the README.</x:v>
+      </x:c>
+      <x:c r="I15" s="14" t="str">
+        <x:v>Code inspection confirms the hero CTA row now includes a Try ATLAS Codex Public Page button, the access-flow panel links to the same public page, and the README contains a dedicated Public ATLAS Codex Page section.</x:v>
+      </x:c>
+      <x:c r="J15" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K15" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L15" s="14" t="str">
+        <x:v>Inspect the hero CTA row and access-flow panel in src/app.js or the built index surface, then inspect README.md for the public ATLAS Codex section and link target.</x:v>
+      </x:c>
+      <x:c r="M15" s="14" t="str">
+        <x:v>Pass - the public ATLAS Codex page is now exposed as a first-class destination from both the site and repo README.</x:v>
+      </x:c>
+      <x:c r="N15" s="14" t="str"/>
+      <x:c r="O15" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P15" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q15" s="14" t="str"/>
+      <x:c r="R15" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S15" s="14" t="str">
+        <x:v>95e35c8</x:v>
+      </x:c>
+      <x:c r="T15" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new CTA row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U15" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after adding the dedicated public ATLAS Codex CTA.</x:v>
+      </x:c>
+      <x:c r="V15" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W15" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X15" s="14" t="str">
+        <x:v>This row captures the stronger direct public ATLAS Codex link requested in the latest pass.</x:v>
+      </x:c>
+      <x:c r="Y15" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="A16" s="14"/>
@@ -12035,7 +12081,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12051,7 +12097,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12115,14 +12161,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record alpha circle conversion pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R34e0d36c7b734ca6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R6a7edaae2a4e4bc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rd7938a3e753c46f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rca04b716f2f54aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R2ce9f20183d54ead"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9932a836032a4ee1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rbff7b49499ae440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R47165b1a69d24af0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1625,85 +1625,223 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
-      <x:c r="A16" s="14"/>
-      <x:c r="B16" s="14"/>
-      <x:c r="C16" s="14"/>
-      <x:c r="D16" s="14"/>
-      <x:c r="E16" s="14"/>
-      <x:c r="F16" s="14"/>
-      <x:c r="G16" s="14"/>
-      <x:c r="H16" s="14"/>
-      <x:c r="I16" s="14"/>
-      <x:c r="J16" s="14"/>
-      <x:c r="K16" s="14"/>
-      <x:c r="L16" s="14"/>
-      <x:c r="M16" s="14"/>
-      <x:c r="N16" s="14"/>
-      <x:c r="O16" s="14"/>
-      <x:c r="P16" s="14"/>
-      <x:c r="Q16" s="14"/>
-      <x:c r="R16" s="14"/>
-      <x:c r="S16" s="14"/>
-      <x:c r="T16" s="14"/>
-      <x:c r="U16" s="14"/>
-      <x:c r="V16" s="14"/>
-      <x:c r="W16" s="14"/>
-      <x:c r="X16" s="14"/>
-      <x:c r="Y16" s="14"/>
+      <x:c r="A16" s="14" t="str">
+        <x:v>F-015</x:v>
+      </x:c>
+      <x:c r="B16" s="14" t="str">
+        <x:v>Alpha Circle Offer Surface</x:v>
+      </x:c>
+      <x:c r="C16" s="14" t="str">
+        <x:v>Membership / Offer</x:v>
+      </x:c>
+      <x:c r="D16" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E16" s="14" t="str">
+        <x:v>Alpha Circle panel and README Alpha Circle section</x:v>
+      </x:c>
+      <x:c r="F16" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G16" s="14" t="str">
+        <x:v>As a prospective Alpha member, I want the public repo to explain what Alpha Circle actually unlocks so that I understand the value behind the join flow.</x:v>
+      </x:c>
+      <x:c r="H16" s="14" t="str">
+        <x:v>The public repo should explain that Alpha Circle unlocks the private ATLAS-7 repo, member-only playbooks, and the deeper MCP operating layer behind the public surface.</x:v>
+      </x:c>
+      <x:c r="I16" s="14" t="str">
+        <x:v>Code inspection confirms the site now includes an Alpha Circle panel with unlock details and the README contains a matching Alpha Circle section.</x:v>
+      </x:c>
+      <x:c r="J16" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K16" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L16" s="14" t="str">
+        <x:v>Inspect the Alpha Circle panel in src/app.js and the Alpha Circle section in README.md for the private repo, member workflow, and MCP unlock explanation.</x:v>
+      </x:c>
+      <x:c r="M16" s="14" t="str">
+        <x:v>Pass - the public repo now explains what Alpha Circle membership unlocks instead of only describing the invite mechanics.</x:v>
+      </x:c>
+      <x:c r="N16" s="14" t="str"/>
+      <x:c r="O16" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P16" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q16" s="14" t="str"/>
+      <x:c r="R16" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S16" s="14" t="str">
+        <x:v>9165df3</x:v>
+      </x:c>
+      <x:c r="T16" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new Alpha Circle row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U16" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after expanding the Alpha Circle public surface.</x:v>
+      </x:c>
+      <x:c r="V16" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W16" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X16" s="14" t="str">
+        <x:v>This row captures the expanded membership offer explanation added in the current pass.</x:v>
+      </x:c>
+      <x:c r="Y16" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
-      <x:c r="A17" s="14"/>
-      <x:c r="B17" s="14"/>
-      <x:c r="C17" s="14"/>
-      <x:c r="D17" s="14"/>
-      <x:c r="E17" s="14"/>
-      <x:c r="F17" s="14"/>
-      <x:c r="G17" s="14"/>
-      <x:c r="H17" s="14"/>
-      <x:c r="I17" s="14"/>
-      <x:c r="J17" s="14"/>
-      <x:c r="K17" s="14"/>
-      <x:c r="L17" s="14"/>
-      <x:c r="M17" s="14"/>
-      <x:c r="N17" s="14"/>
-      <x:c r="O17" s="14"/>
-      <x:c r="P17" s="14"/>
-      <x:c r="Q17" s="14"/>
-      <x:c r="R17" s="14"/>
-      <x:c r="S17" s="14"/>
-      <x:c r="T17" s="14"/>
-      <x:c r="U17" s="14"/>
-      <x:c r="V17" s="14"/>
-      <x:c r="W17" s="14"/>
-      <x:c r="X17" s="14"/>
-      <x:c r="Y17" s="14"/>
+      <x:c r="A17" s="14" t="str">
+        <x:v>F-016</x:v>
+      </x:c>
+      <x:c r="B17" s="14" t="str">
+        <x:v>Referral System Surface</x:v>
+      </x:c>
+      <x:c r="C17" s="14" t="str">
+        <x:v>Membership / Referral</x:v>
+      </x:c>
+      <x:c r="D17" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E17" s="14" t="str">
+        <x:v>Referral System panel and README referral section</x:v>
+      </x:c>
+      <x:c r="F17" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G17" s="14" t="str">
+        <x:v>As a serious operator considering Alpha, I want the referral rules explained so that I know how the MCP credit incentive works and what kind of referral counts.</x:v>
+      </x:c>
+      <x:c r="H17" s="14" t="str">
+        <x:v>The public repo should explain that referrals count when the referred person becomes an Alpha Circle member and that founding-member referrals can earn additional MCP credits.</x:v>
+      </x:c>
+      <x:c r="I17" s="14" t="str">
+        <x:v>Code inspection confirms the site now includes a Referral System panel and the README contains a matching referral section covering Alpha-member conversion and MCP credit language.</x:v>
+      </x:c>
+      <x:c r="J17" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K17" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L17" s="14" t="str">
+        <x:v>Inspect the Referral System panel in src/app.js and the Referral System section in README.md for Alpha-member conversion and MCP credit messaging.</x:v>
+      </x:c>
+      <x:c r="M17" s="14" t="str">
+        <x:v>Pass - the referral loop is now visible on both the site and README instead of being left implicit.</x:v>
+      </x:c>
+      <x:c r="N17" s="14" t="str"/>
+      <x:c r="O17" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P17" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q17" s="14" t="str"/>
+      <x:c r="R17" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S17" s="14" t="str">
+        <x:v>9165df3</x:v>
+      </x:c>
+      <x:c r="T17" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new referral row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U17" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after expanding the Alpha Circle public surface.</x:v>
+      </x:c>
+      <x:c r="V17" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W17" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X17" s="14" t="str">
+        <x:v>This row captures the public referral-system explanation requested in the current pass.</x:v>
+      </x:c>
+      <x:c r="Y17" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
-      <x:c r="A18" s="14"/>
-      <x:c r="B18" s="14"/>
-      <x:c r="C18" s="14"/>
-      <x:c r="D18" s="14"/>
-      <x:c r="E18" s="14"/>
-      <x:c r="F18" s="14"/>
-      <x:c r="G18" s="14"/>
-      <x:c r="H18" s="14"/>
-      <x:c r="I18" s="14"/>
-      <x:c r="J18" s="14"/>
-      <x:c r="K18" s="14"/>
-      <x:c r="L18" s="14"/>
-      <x:c r="M18" s="14"/>
-      <x:c r="N18" s="14"/>
-      <x:c r="O18" s="14"/>
-      <x:c r="P18" s="14"/>
-      <x:c r="Q18" s="14"/>
-      <x:c r="R18" s="14"/>
-      <x:c r="S18" s="14"/>
-      <x:c r="T18" s="14"/>
-      <x:c r="U18" s="14"/>
-      <x:c r="V18" s="14"/>
-      <x:c r="W18" s="14"/>
-      <x:c r="X18" s="14"/>
-      <x:c r="Y18" s="14"/>
+      <x:c r="A18" s="14" t="str">
+        <x:v>F-017</x:v>
+      </x:c>
+      <x:c r="B18" s="14" t="str">
+        <x:v>Substack Join Links</x:v>
+      </x:c>
+      <x:c r="C18" s="14" t="str">
+        <x:v>Membership / External Navigation</x:v>
+      </x:c>
+      <x:c r="D18" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E18" s="14" t="str">
+        <x:v>Join Links panel, access-flow helper copy, README join links section</x:v>
+      </x:c>
+      <x:c r="F18" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G18" s="14" t="str">
+        <x:v>As a prospective member, I want the exact DeltaSignal and Alpha Circle note links so that I know where to subscribe and where to read the public explanation before joining.</x:v>
+      </x:c>
+      <x:c r="H18" s="14" t="str">
+        <x:v>The public repo should link directly to the DeltaSignal Substack home and the Alpha Circle note in both the site and README.</x:v>
+      </x:c>
+      <x:c r="I18" s="14" t="str">
+        <x:v>Code inspection confirms the site now exposes both the DeltaSignal Substack and Alpha Circle note links in the Join Links panel and access-flow copy, and the README contains the same join links.</x:v>
+      </x:c>
+      <x:c r="J18" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K18" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L18" s="14" t="str">
+        <x:v>Inspect the Join Links panel and access-flow copy in src/app.js, then inspect README.md for the Join Links section and exact targets.</x:v>
+      </x:c>
+      <x:c r="M18" s="14" t="str">
+        <x:v>Pass - the exact Substack entry points for joining and reading the note are now explicit in both site and README.</x:v>
+      </x:c>
+      <x:c r="N18" s="14" t="str"/>
+      <x:c r="O18" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P18" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q18" s="14" t="str"/>
+      <x:c r="R18" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S18" s="14" t="str">
+        <x:v>9165df3</x:v>
+      </x:c>
+      <x:c r="T18" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new Substack links row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U18" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after expanding the Alpha Circle public surface.</x:v>
+      </x:c>
+      <x:c r="V18" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W18" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X18" s="14" t="str">
+        <x:v>This row captures the explicit DeltaSignal and Alpha Circle note links added in the current pass.</x:v>
+      </x:c>
+      <x:c r="Y18" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="14"/>
@@ -12081,7 +12219,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12097,7 +12235,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12161,14 +12299,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record join handoff clarity pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R2ce9f20183d54ead"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9932a836032a4ee1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rbff7b49499ae440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R47165b1a69d24af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Ree3148a5fd9e4321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R95e3f7b0aaf54c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R2028ffdb3ee548af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R84600a3de069482b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1844,31 +1844,77 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
-      <x:c r="A19" s="14"/>
-      <x:c r="B19" s="14"/>
-      <x:c r="C19" s="14"/>
-      <x:c r="D19" s="14"/>
-      <x:c r="E19" s="14"/>
-      <x:c r="F19" s="14"/>
-      <x:c r="G19" s="14"/>
-      <x:c r="H19" s="14"/>
-      <x:c r="I19" s="14"/>
-      <x:c r="J19" s="14"/>
-      <x:c r="K19" s="14"/>
-      <x:c r="L19" s="14"/>
-      <x:c r="M19" s="14"/>
-      <x:c r="N19" s="14"/>
-      <x:c r="O19" s="14"/>
-      <x:c r="P19" s="14"/>
-      <x:c r="Q19" s="14"/>
-      <x:c r="R19" s="14"/>
-      <x:c r="S19" s="14"/>
-      <x:c r="T19" s="14"/>
-      <x:c r="U19" s="14"/>
-      <x:c r="V19" s="14"/>
-      <x:c r="W19" s="14"/>
-      <x:c r="X19" s="14"/>
-      <x:c r="Y19" s="14"/>
+      <x:c r="A19" s="14" t="str">
+        <x:v>F-018</x:v>
+      </x:c>
+      <x:c r="B19" s="14" t="str">
+        <x:v>Join Handoff Clarity</x:v>
+      </x:c>
+      <x:c r="C19" s="14" t="str">
+        <x:v>Membership / Access Copy</x:v>
+      </x:c>
+      <x:c r="D19" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E19" s="14" t="str">
+        <x:v>Hero join strip, access-flow list, README join section</x:v>
+      </x:c>
+      <x:c r="F19" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G19" s="14" t="str">
+        <x:v>As a prospective member, I want the join handoff explained in simple bullets so that I know exactly where to join and where to send my GitHub details.</x:v>
+      </x:c>
+      <x:c r="H19" s="14" t="str">
+        <x:v>The public repo should present the join flow as bullets, include the direct Alpha link, and state that the GitHub username or account email should be sent by replying to DeltaSignal after joining.</x:v>
+      </x:c>
+      <x:c r="I19" s="14" t="str">
+        <x:v>Code inspection confirms the hero join strip now uses bullets, the access-flow list includes the direct Alpha link, and the README mirrors the same bullet-based handoff language.</x:v>
+      </x:c>
+      <x:c r="J19" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K19" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L19" s="14" t="str">
+        <x:v>Inspect the hero join strip and access-flow list in src/app.js, then inspect README.md for the matching bullet-based join handoff copy.</x:v>
+      </x:c>
+      <x:c r="M19" s="14" t="str">
+        <x:v>Pass - the join flow is now bullet-based, linked, and explicit about replying to DeltaSignal after joining.</x:v>
+      </x:c>
+      <x:c r="N19" s="14" t="str"/>
+      <x:c r="O19" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P19" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q19" s="14" t="str"/>
+      <x:c r="R19" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S19" s="14" t="str">
+        <x:v>4b525f3</x:v>
+      </x:c>
+      <x:c r="T19" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new join-handoff row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U19" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after clarifying the join handoff copy.</x:v>
+      </x:c>
+      <x:c r="V19" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W19" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X19" s="14" t="str">
+        <x:v>This row captures the clearer bullet-based join handoff requested in the latest pass.</x:v>
+      </x:c>
+      <x:c r="Y19" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="14"/>
@@ -12219,7 +12265,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12235,7 +12281,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12299,14 +12345,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record alpha guide link pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R56e83c32525d4fe6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb32be5526ed94f00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R8965438b62744d8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R3d6d8cfeaf1346d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rb8d8a4a48f2e4e82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5844e1a13cc44ae1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rb9a8e0d939904b11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R9094e3314b904895"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2063,31 +2063,77 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="14"/>
-      <x:c r="B22" s="14"/>
-      <x:c r="C22" s="14"/>
-      <x:c r="D22" s="14"/>
-      <x:c r="E22" s="14"/>
-      <x:c r="F22" s="14"/>
-      <x:c r="G22" s="14"/>
-      <x:c r="H22" s="14"/>
-      <x:c r="I22" s="14"/>
-      <x:c r="J22" s="14"/>
-      <x:c r="K22" s="14"/>
-      <x:c r="L22" s="14"/>
-      <x:c r="M22" s="14"/>
-      <x:c r="N22" s="14"/>
-      <x:c r="O22" s="14"/>
-      <x:c r="P22" s="14"/>
-      <x:c r="Q22" s="14"/>
-      <x:c r="R22" s="14"/>
-      <x:c r="S22" s="14"/>
-      <x:c r="T22" s="14"/>
-      <x:c r="U22" s="14"/>
-      <x:c r="V22" s="14"/>
-      <x:c r="W22" s="14"/>
-      <x:c r="X22" s="14"/>
-      <x:c r="Y22" s="14"/>
+      <x:c r="A22" s="14" t="str">
+        <x:v>F-021</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>Alpha Circle Join Guide As Primary Link</x:v>
+      </x:c>
+      <x:c r="C22" s="14" t="str">
+        <x:v>Membership / Conversion</x:v>
+      </x:c>
+      <x:c r="D22" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E22" s="14" t="str">
+        <x:v>Hero primary CTA, join strip, join links panel, access-flow panel, README access section</x:v>
+      </x:c>
+      <x:c r="F22" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G22" s="14" t="str">
+        <x:v>As a prospective member, I want the main Alpha link to land on the exact join guide so that I get the most direct explanation of how to become an Alpha Circle member.</x:v>
+      </x:c>
+      <x:c r="H22" s="14" t="str">
+        <x:v>The public repo should use the Alpha Circle note URL as the primary join destination in the main CTA and the step-by-step access instructions, while keeping the broader DeltaSignal Substack available as a secondary link.</x:v>
+      </x:c>
+      <x:c r="I22" s="14" t="str">
+        <x:v>Code inspection confirms the hero CTA, join strip, join links panel, access-flow panel, and README now use the Alpha Circle note as the primary join destination and keep DeltaSignal Substack as a secondary supporting link.</x:v>
+      </x:c>
+      <x:c r="J22" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K22" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L22" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the primary Alpha-link targets and confirm the join-guide URL is now the main membership destination.</x:v>
+      </x:c>
+      <x:c r="M22" s="14" t="str">
+        <x:v>Pass - the public repo now points its main conversion path to the exact Alpha Circle join guide instead of the broader home page.</x:v>
+      </x:c>
+      <x:c r="N22" s="14" t="str"/>
+      <x:c r="O22" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P22" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q22" s="14" t="str"/>
+      <x:c r="R22" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S22" s="14" t="str">
+        <x:v>a3b3e47</x:v>
+      </x:c>
+      <x:c r="T22" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new primary-link row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U22" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after retargeting the main Alpha join path to the dedicated join guide.</x:v>
+      </x:c>
+      <x:c r="V22" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W22" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X22" s="14" t="str">
+        <x:v>This row captures the retargeting of the public repo's main Alpha join path to the dedicated Alpha Circle guide.</x:v>
+      </x:c>
+      <x:c r="Y22" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="14"/>
@@ -12357,7 +12403,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12373,7 +12419,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12437,14 +12483,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record contents anchor pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R71f743c708424a6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9fd296f6f2f84d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R12ad10fc83184776"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rf3d9ce375fc140ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rf8f12ba5d0284430"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rcb8c2c91876f4b57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rf873444b96e544d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R421ea8b4f1174600"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2428,31 +2428,77 @@
       </x:c>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="14"/>
-      <x:c r="B27" s="14"/>
-      <x:c r="C27" s="14"/>
-      <x:c r="D27" s="14"/>
-      <x:c r="E27" s="14"/>
-      <x:c r="F27" s="14"/>
-      <x:c r="G27" s="14"/>
-      <x:c r="H27" s="14"/>
-      <x:c r="I27" s="14"/>
-      <x:c r="J27" s="14"/>
-      <x:c r="K27" s="14"/>
-      <x:c r="L27" s="14"/>
-      <x:c r="M27" s="14"/>
-      <x:c r="N27" s="14"/>
-      <x:c r="O27" s="14"/>
-      <x:c r="P27" s="14"/>
-      <x:c r="Q27" s="14"/>
-      <x:c r="R27" s="14"/>
-      <x:c r="S27" s="14"/>
-      <x:c r="T27" s="14"/>
-      <x:c r="U27" s="14"/>
-      <x:c r="V27" s="14"/>
-      <x:c r="W27" s="14"/>
-      <x:c r="X27" s="14"/>
-      <x:c r="Y27" s="14"/>
+      <x:c r="A27" s="14" t="str">
+        <x:v>F-026</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>Contents Anchor Navigation</x:v>
+      </x:c>
+      <x:c r="C27" s="14" t="str">
+        <x:v>Navigation / In-Page</x:v>
+      </x:c>
+      <x:c r="D27" s="14" t="str">
+        <x:v>src/app.js</x:v>
+      </x:c>
+      <x:c r="E27" s="14" t="str">
+        <x:v>Contents panel links to section anchors</x:v>
+      </x:c>
+      <x:c r="F27" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G27" s="14" t="str">
+        <x:v>As a visitor, I want the Contents links to land on the intended sections so that I can jump directly to the right part of the page.</x:v>
+      </x:c>
+      <x:c r="H27" s="14" t="str">
+        <x:v>The Contents links should scroll to the matching in-page sections inside the Lit app instead of relying on default fragment behavior that may miss shadow-root content.</x:v>
+      </x:c>
+      <x:c r="I27" s="14" t="str">
+        <x:v>Code inspection confirms the Contents links now call an in-component scroll handler, use `scrollIntoView`, and target the matching section ids directly.</x:v>
+      </x:c>
+      <x:c r="J27" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K27" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L27" s="14" t="str">
+        <x:v>Inspect src/app.js for the Contents link click handlers and the in-component target lookup, then confirm the section ids still match the link targets.</x:v>
+      </x:c>
+      <x:c r="M27" s="14" t="str">
+        <x:v>Pass - the Contents links are now wired to explicit in-page scrolling for the correct sections.</x:v>
+      </x:c>
+      <x:c r="N27" s="14" t="str"/>
+      <x:c r="O27" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P27" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q27" s="14" t="str"/>
+      <x:c r="R27" s="14" t="str">
+        <x:v>src/app.js, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S27" s="14" t="str">
+        <x:v>fc7c543</x:v>
+      </x:c>
+      <x:c r="T27" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new contents-anchor row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U27" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after wiring explicit Contents scrolling inside the Lit page.</x:v>
+      </x:c>
+      <x:c r="V27" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W27" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X27" s="14" t="str">
+        <x:v>This row captures the fix for Contents navigation inside the Lit shadow-root page.</x:v>
+      </x:c>
+      <x:c r="Y27" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="14"/>
@@ -12587,7 +12633,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12603,7 +12649,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12667,14 +12713,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record scarcity framing pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R4d3de0ff9ed4441d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R17c83812e3684e5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Re0388b8b2d594e2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Ra61978f1955f4ef2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rea3d7a1542314d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R3067fd68c8ac42f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R991255192d73451d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R795cda8671e44288"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2574,31 +2574,77 @@
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="14"/>
-      <x:c r="B29" s="14"/>
-      <x:c r="C29" s="14"/>
-      <x:c r="D29" s="14"/>
-      <x:c r="E29" s="14"/>
-      <x:c r="F29" s="14"/>
-      <x:c r="G29" s="14"/>
-      <x:c r="H29" s="14"/>
-      <x:c r="I29" s="14"/>
-      <x:c r="J29" s="14"/>
-      <x:c r="K29" s="14"/>
-      <x:c r="L29" s="14"/>
-      <x:c r="M29" s="14"/>
-      <x:c r="N29" s="14"/>
-      <x:c r="O29" s="14"/>
-      <x:c r="P29" s="14"/>
-      <x:c r="Q29" s="14"/>
-      <x:c r="R29" s="14"/>
-      <x:c r="S29" s="14"/>
-      <x:c r="T29" s="14"/>
-      <x:c r="U29" s="14"/>
-      <x:c r="V29" s="14"/>
-      <x:c r="W29" s="14"/>
-      <x:c r="X29" s="14"/>
-      <x:c r="Y29" s="14"/>
+      <x:c r="A29" s="14" t="str">
+        <x:v>F-028</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>Scarcity And Selective Access Framing</x:v>
+      </x:c>
+      <x:c r="C29" s="14" t="str">
+        <x:v>Marketing / Conversion Copy</x:v>
+      </x:c>
+      <x:c r="D29" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E29" s="14" t="str">
+        <x:v>Hero CTA, limited-access copy, Alpha section, README access framing</x:v>
+      </x:c>
+      <x:c r="F29" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G29" s="14" t="str">
+        <x:v>As a prospective member, I want the page to communicate scarcity and selective access so that the Alpha Circle offer feels more clearly differentiated and time-sensitive.</x:v>
+      </x:c>
+      <x:c r="H29" s="14" t="str">
+        <x:v>The public landing page should add limited-access framing, a stronger join CTA, and selective-membership language while preserving the existing join flow and GitHub handoff steps.</x:v>
+      </x:c>
+      <x:c r="I29" s="14" t="str">
+        <x:v>Code inspection confirms the hero CTA, limited-access copy, landing-page sections, and README now include scarcity and selective-membership framing around Alpha Circle access.</x:v>
+      </x:c>
+      <x:c r="J29" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K29" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L29" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the stronger CTA, limited-access section, and selective-membership copy.</x:v>
+      </x:c>
+      <x:c r="M29" s="14" t="str">
+        <x:v>Pass - the public page now frames Alpha Circle access as intentionally limited while keeping the same practical join path.</x:v>
+      </x:c>
+      <x:c r="N29" s="14" t="str"/>
+      <x:c r="O29" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P29" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q29" s="14" t="str"/>
+      <x:c r="R29" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S29" s="14" t="str">
+        <x:v>f3eef44</x:v>
+      </x:c>
+      <x:c r="T29" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new scarcity row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U29" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after adding scarcity and selective-membership framing to the public page.</x:v>
+      </x:c>
+      <x:c r="V29" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W29" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X29" s="14" t="str">
+        <x:v>This row captures the scarcity-oriented marketing pass for the public landing page.</x:v>
+      </x:c>
+      <x:c r="Y29" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="14"/>
@@ -12679,7 +12725,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12695,7 +12741,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12759,14 +12805,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>